<commit_message>
added link to COMP560 Team on Microsoft Teams
</commit_message>
<xml_diff>
--- a/comp560-schedule-7-31-2026.xlsx
+++ b/comp560-schedule-7-31-2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jmac\git\comp560-web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="513" documentId="13_ncr:1_{91DEECA4-1339-44A4-B91E-F265F67426BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{514F9B28-FA0A-490A-9E70-97696106FA3B}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7470CF8-7EAB-4461-8C94-0327625ABBA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="9540" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -609,6 +609,15 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -631,15 +640,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -976,10 +976,10 @@
       <c r="F1" s="5"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="35" t="s">
+      <c r="A2" s="38" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="38" t="s">
+      <c r="B2" s="30" t="s">
         <v>1</v>
       </c>
       <c r="C2" s="23">
@@ -990,8 +990,8 @@
       <c r="F2" s="7"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="36"/>
-      <c r="B3" s="39"/>
+      <c r="A3" s="39"/>
+      <c r="B3" s="32"/>
       <c r="C3" s="3">
         <v>46267</v>
       </c>
@@ -1002,8 +1002,8 @@
       <c r="F3" s="7"/>
     </row>
     <row r="4" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="36"/>
-      <c r="B4" s="40"/>
+      <c r="A4" s="39"/>
+      <c r="B4" s="31"/>
       <c r="C4" s="15">
         <v>46273</v>
       </c>
@@ -1014,8 +1014,8 @@
       <c r="F4" s="7"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="36"/>
-      <c r="B5" s="38" t="s">
+      <c r="A5" s="39"/>
+      <c r="B5" s="30" t="s">
         <v>2</v>
       </c>
       <c r="C5" s="23">
@@ -1028,8 +1028,8 @@
       <c r="F5" s="7"/>
     </row>
     <row r="6" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="36"/>
-      <c r="B6" s="40"/>
+      <c r="A6" s="39"/>
+      <c r="B6" s="31"/>
       <c r="C6" s="15">
         <f>C5+6</f>
         <v>46280</v>
@@ -1041,8 +1041,8 @@
       <c r="F6" s="7"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="36"/>
-      <c r="B7" s="38" t="s">
+      <c r="A7" s="39"/>
+      <c r="B7" s="30" t="s">
         <v>3</v>
       </c>
       <c r="C7" s="23">
@@ -1056,8 +1056,8 @@
       <c r="F7" s="7"/>
     </row>
     <row r="8" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="37"/>
-      <c r="B8" s="40"/>
+      <c r="A8" s="40"/>
+      <c r="B8" s="31"/>
       <c r="C8" s="15">
         <f t="shared" ref="C8" si="0">C7+6</f>
         <v>46287</v>
@@ -1069,10 +1069,10 @@
       <c r="F8" s="7"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="35" t="s">
+      <c r="A9" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="38" t="s">
+      <c r="B9" s="30" t="s">
         <v>4</v>
       </c>
       <c r="C9" s="23">
@@ -1086,8 +1086,8 @@
       <c r="F9" s="7"/>
     </row>
     <row r="10" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="36"/>
-      <c r="B10" s="40"/>
+      <c r="A10" s="39"/>
+      <c r="B10" s="31"/>
       <c r="C10" s="15">
         <f t="shared" ref="C10" si="2">C9+6</f>
         <v>46294</v>
@@ -1099,8 +1099,8 @@
       <c r="F10" s="7"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="36"/>
-      <c r="B11" s="38" t="s">
+      <c r="A11" s="39"/>
+      <c r="B11" s="30" t="s">
         <v>5</v>
       </c>
       <c r="C11" s="23">
@@ -1114,8 +1114,8 @@
       <c r="F11" s="7"/>
     </row>
     <row r="12" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="36"/>
-      <c r="B12" s="40"/>
+      <c r="A12" s="39"/>
+      <c r="B12" s="31"/>
       <c r="C12" s="15">
         <f t="shared" ref="C12" si="4">C11+6</f>
         <v>46301</v>
@@ -1127,8 +1127,8 @@
       <c r="F12" s="7"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="36"/>
-      <c r="B13" s="38" t="s">
+      <c r="A13" s="39"/>
+      <c r="B13" s="30" t="s">
         <v>6</v>
       </c>
       <c r="C13" s="23">
@@ -1142,8 +1142,8 @@
       <c r="F13" s="7"/>
     </row>
     <row r="14" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="37"/>
-      <c r="B14" s="40"/>
+      <c r="A14" s="40"/>
+      <c r="B14" s="31"/>
       <c r="C14" s="15">
         <f t="shared" ref="C14:C28" si="6">C13+6</f>
         <v>46308</v>
@@ -1155,10 +1155,10 @@
       <c r="F14" s="7"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="35" t="s">
+      <c r="A15" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="38" t="s">
+      <c r="B15" s="30" t="s">
         <v>7</v>
       </c>
       <c r="C15" s="23">
@@ -1172,21 +1172,21 @@
       <c r="F15" s="7"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="36"/>
-      <c r="B16" s="39"/>
+      <c r="A16" s="39"/>
+      <c r="B16" s="32"/>
       <c r="C16" s="3">
         <f t="shared" si="6"/>
         <v>46315</v>
       </c>
-      <c r="D16" s="30" t="s">
+      <c r="D16" s="33" t="s">
         <v>44</v>
       </c>
-      <c r="E16" s="31"/>
+      <c r="E16" s="34"/>
       <c r="F16" s="10"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="36"/>
-      <c r="B17" s="39"/>
+      <c r="A17" s="39"/>
+      <c r="B17" s="32"/>
       <c r="C17" s="3">
         <f t="shared" si="5"/>
         <v>46316</v>
@@ -1198,8 +1198,8 @@
       <c r="F17" s="7"/>
     </row>
     <row r="18" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="36"/>
-      <c r="B18" s="40"/>
+      <c r="A18" s="39"/>
+      <c r="B18" s="31"/>
       <c r="C18" s="15">
         <f t="shared" si="6"/>
         <v>46322</v>
@@ -1211,8 +1211,8 @@
       <c r="F18" s="7"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="36"/>
-      <c r="B19" s="38" t="s">
+      <c r="A19" s="39"/>
+      <c r="B19" s="30" t="s">
         <v>8</v>
       </c>
       <c r="C19" s="23">
@@ -1226,8 +1226,8 @@
       <c r="F19" s="7"/>
     </row>
     <row r="20" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="36"/>
-      <c r="B20" s="40"/>
+      <c r="A20" s="39"/>
+      <c r="B20" s="31"/>
       <c r="C20" s="15">
         <f t="shared" si="6"/>
         <v>46329</v>
@@ -1239,8 +1239,8 @@
       <c r="F20" s="7"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="36"/>
-      <c r="B21" s="38" t="s">
+      <c r="A21" s="39"/>
+      <c r="B21" s="30" t="s">
         <v>9</v>
       </c>
       <c r="C21" s="23">
@@ -1254,8 +1254,8 @@
       <c r="F21" s="7"/>
     </row>
     <row r="22" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="37"/>
-      <c r="B22" s="40"/>
+      <c r="A22" s="40"/>
+      <c r="B22" s="31"/>
       <c r="C22" s="15">
         <f t="shared" si="6"/>
         <v>46336</v>
@@ -1267,10 +1267,10 @@
       <c r="F22" s="7"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" s="35" t="s">
+      <c r="A23" s="38" t="s">
         <v>16</v>
       </c>
-      <c r="B23" s="38" t="s">
+      <c r="B23" s="30" t="s">
         <v>10</v>
       </c>
       <c r="C23" s="23">
@@ -1284,8 +1284,8 @@
       <c r="F23" s="7"/>
     </row>
     <row r="24" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="36"/>
-      <c r="B24" s="40"/>
+      <c r="A24" s="39"/>
+      <c r="B24" s="31"/>
       <c r="C24" s="15">
         <f t="shared" si="6"/>
         <v>46343</v>
@@ -1297,8 +1297,8 @@
       <c r="F24" s="7"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25" s="36"/>
-      <c r="B25" s="38" t="s">
+      <c r="A25" s="39"/>
+      <c r="B25" s="30" t="s">
         <v>11</v>
       </c>
       <c r="C25" s="23">
@@ -1312,8 +1312,8 @@
       <c r="F25" s="7"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A26" s="36"/>
-      <c r="B26" s="39"/>
+      <c r="A26" s="39"/>
+      <c r="B26" s="32"/>
       <c r="C26" s="3">
         <f t="shared" si="6"/>
         <v>46350</v>
@@ -1323,21 +1323,21 @@
       <c r="F26" s="7"/>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A27" s="36"/>
-      <c r="B27" s="39"/>
+      <c r="A27" s="39"/>
+      <c r="B27" s="32"/>
       <c r="C27" s="3">
         <f t="shared" si="5"/>
         <v>46351</v>
       </c>
-      <c r="D27" s="30" t="s">
+      <c r="D27" s="33" t="s">
         <v>39</v>
       </c>
-      <c r="E27" s="31"/>
+      <c r="E27" s="34"/>
       <c r="F27" s="10"/>
     </row>
     <row r="28" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="36"/>
-      <c r="B28" s="40"/>
+      <c r="A28" s="39"/>
+      <c r="B28" s="31"/>
       <c r="C28" s="15">
         <f t="shared" si="6"/>
         <v>46357</v>
@@ -1349,8 +1349,8 @@
       <c r="F28" s="7"/>
     </row>
     <row r="29" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="36"/>
-      <c r="B29" s="32" t="s">
+      <c r="A29" s="39"/>
+      <c r="B29" s="35" t="s">
         <v>12</v>
       </c>
       <c r="C29" s="23">
@@ -1364,8 +1364,8 @@
       <c r="F29" s="11"/>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A30" s="36"/>
-      <c r="B30" s="33"/>
+      <c r="A30" s="39"/>
+      <c r="B30" s="36"/>
       <c r="C30" s="3">
         <f>C29+1</f>
         <v>46359</v>
@@ -1377,8 +1377,8 @@
       <c r="F30" s="7"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A31" s="36"/>
-      <c r="B31" s="33"/>
+      <c r="A31" s="39"/>
+      <c r="B31" s="36"/>
       <c r="C31" s="3">
         <f t="shared" si="5"/>
         <v>46365</v>
@@ -1390,8 +1390,8 @@
       <c r="F31" s="7"/>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A32" s="36"/>
-      <c r="B32" s="33"/>
+      <c r="A32" s="39"/>
+      <c r="B32" s="36"/>
       <c r="C32" s="3">
         <f>C31+2</f>
         <v>46367</v>
@@ -1400,8 +1400,8 @@
       <c r="F32" s="7"/>
     </row>
     <row r="33" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="37"/>
-      <c r="B33" s="34"/>
+      <c r="A33" s="40"/>
+      <c r="B33" s="37"/>
       <c r="C33" s="15">
         <v>46375</v>
       </c>
@@ -1412,11 +1412,6 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="B23:B24"/>
-    <mergeCell ref="B25:B28"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="B29:B33"/>
     <mergeCell ref="A2:A8"/>
     <mergeCell ref="A9:A14"/>
     <mergeCell ref="A15:A22"/>
@@ -1430,6 +1425,11 @@
     <mergeCell ref="B15:B18"/>
     <mergeCell ref="B19:B20"/>
     <mergeCell ref="B21:B22"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="B25:B28"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="B29:B33"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>